<commit_message>
Submit complete assignment folder updates
</commit_message>
<xml_diff>
--- a/DN - Java FSE Mandatory hands-on detail.xlsx
+++ b/DN - Java FSE Mandatory hands-on detail.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91985\Desktop\Asgns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29566D7-84F5-42B4-BA69-353EF67F6AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C20D3A6-BF91-4D93-A6A2-4526A155932D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E078EC40-2268-4F4F-B14B-9403122955B8}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="95">
   <si>
     <t>Skill</t>
   </si>
@@ -340,7 +340,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -367,13 +367,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0070C0"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -563,8 +557,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -597,6 +589,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -942,21 +936,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="27" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="E1" s="28"/>
+      <c r="E1" s="26"/>
       <c r="F1" s="8"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="20"/>
+      <c r="A2" s="18"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1103,29 +1097,29 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="21" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="29"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="27"/>
       <c r="F11" s="14" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="24"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="22"/>
       <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="30"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="28"/>
       <c r="F12" s="14" t="s">
         <v>94</v>
       </c>
@@ -1343,7 +1337,7 @@
       <c r="B25" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="30" t="s">
         <v>48</v>
       </c>
       <c r="D25" s="4" t="s">
@@ -1363,7 +1357,7 @@
       <c r="B26" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="30" t="s">
         <v>51</v>
       </c>
       <c r="D26" s="4"/>
@@ -1379,7 +1373,7 @@
       <c r="B27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="30" t="s">
         <v>53</v>
       </c>
       <c r="D27" s="4"/>
@@ -1395,7 +1389,7 @@
       <c r="B28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D28" s="4"/>
@@ -1411,7 +1405,7 @@
       <c r="B29" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="30" t="s">
         <v>55</v>
       </c>
       <c r="D29" s="4"/>
@@ -1437,16 +1431,16 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="19" t="s">
         <v>59</v>
       </c>
       <c r="E31" s="11" t="s">
@@ -1457,10 +1451,10 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="22"/>
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="22"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="20"/>
       <c r="E32" s="12" t="s">
         <v>62</v>
       </c>
@@ -1616,7 +1610,9 @@
       <c r="E40" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="F40" s="8"/>
+      <c r="F40" s="14" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
@@ -1634,7 +1630,9 @@
       <c r="E41" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="F41" s="8"/>
+      <c r="F41" s="14" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
@@ -1652,7 +1650,9 @@
       <c r="E42" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="F42" s="8"/>
+      <c r="F42" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
@@ -1666,7 +1666,9 @@
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="10"/>
-      <c r="F43" s="8"/>
+      <c r="F43" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
@@ -1680,7 +1682,9 @@
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="10"/>
-      <c r="F44" s="8"/>
+      <c r="F44" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
@@ -1694,7 +1698,9 @@
       </c>
       <c r="D45" s="4"/>
       <c r="E45" s="10"/>
-      <c r="F45" s="8"/>
+      <c r="F45" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
@@ -1708,7 +1714,9 @@
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="10"/>
-      <c r="F46" s="8"/>
+      <c r="F46" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
@@ -1722,7 +1730,9 @@
       </c>
       <c r="D47" s="4"/>
       <c r="E47" s="10"/>
-      <c r="F47" s="8"/>
+      <c r="F47" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
@@ -1736,7 +1746,9 @@
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="13"/>
-      <c r="F48" s="8"/>
+      <c r="F48" s="29" t="s">
+        <v>94</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1757,15 +1769,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6f516c4-2602-422c-aa9a-755893ba4f98">
@@ -1774,6 +1777,15 @@
     <TaxCatchAll xmlns="3c35e321-f73a-4dae-ae38-a0459de24735"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2037,14 +2049,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F0F638-0648-46BA-B1DF-3E4F6ADB00E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B84191-BBE7-412A-A5F6-7B8D27AECA6C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -2058,6 +2062,14 @@
     <ds:schemaRef ds:uri="951c5514-b77c-4532-82d5-a05f2f7d58e2"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F0F638-0648-46BA-B1DF-3E4F6ADB00E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>